<commit_message>
feat: add exact-one-face gate and sync docs
</commit_message>
<xml_diff>
--- a/frontend/public/gen-sticker-docs/originals/02-prd.xlsx
+++ b/frontend/public/gen-sticker-docs/originals/02-prd.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visual User Journey" sheetId="1" r:id="R3200f7797e3e4d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R57153ad237f3497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra4dcd1940dd24236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Flows" sheetId="4" r:id="R5211a37c18324164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limits &amp; KPI" sheetId="5" r:id="R4df9f7bb01cf49cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions &amp; Gaps" sheetId="6" r:id="R38fc21d1fe0a4781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Dashboard" sheetId="7" r:id="R8231bc26ba144681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholders" sheetId="8" r:id="Rdc7eb09b41884a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Criteria" sheetId="9" r:id="R994645bdaa9047ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="10" r:id="R6597df5122994764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics Plan" sheetId="11" r:id="R6cf14fc778884313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visual User Journey" sheetId="1" r:id="Rf83cd920df194b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R03b1f95ec61e40a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R02cfd9eea23340ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Flows" sheetId="4" r:id="R27aed2a67dd84329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limits &amp; KPI" sheetId="5" r:id="Rc2e82a0f9dfc4e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions &amp; Gaps" sheetId="6" r:id="Re7ca59fe279f4b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Dashboard" sheetId="7" r:id="R5318a09f450e4346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholders" sheetId="8" r:id="R5e976ded83024e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Criteria" sheetId="9" r:id="R4c05fdb343904828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="10" r:id="Rfab684ef651b4280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics Plan" sheetId="11" r:id="R02e387c26a9f4b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Face Gate Requirements" sheetId="12" r:id="R1116f8a2bd934436"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +521,7 @@
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:rPr sz="975"/>
-              <a:t>14 requirements by implementation status</a:t>
+              <a:t>15 requirements by implementation status</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -593,13 +594,13 @@
     <xdr:ext cx="11734800" cy="6600825"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="56986284-5867-4539-b971-905a943bf382"/>
+        <xdr:cNvPr id="1" name="72ace3ba-c0bc-43d3-a1ad-61eacaaca7ec"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf28b88d5177e407e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2a50aaccaee54c38"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -639,7 +640,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48693096a7084f31"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4d938818ecf346f3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -674,9 +675,23 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="GS0211Table" displayName="GS0211Table" ref="A6:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:E13"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Requirement"/>
+    <x:tableColumn id="3" name="Acceptance"/>
+    <x:tableColumn id="4" name="Status"/>
+    <x:tableColumn id="5" name="Evidence"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GS0202Table" displayName="GS0202Table" ref="A6:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GS0202Table" displayName="GS0202Table" ref="A6:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H21"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nhóm"/>
@@ -1019,7 +1034,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Luồng UI thực tế trên kien_v5, gồm auth, polling và rejected state</x:v>
+        <x:v>Face preflight cục bộ đứng trước job và mọi image call trả phí</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1071,7 +1086,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16" t="str">
-        <x:v>Luồng từ chọn ảnh, xác thực, tạo job, polling đến gallery</x:v>
+        <x:v>Luồng chọn ảnh qua Web Worker MediaPipe</x:v>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>
@@ -1079,7 +1094,7 @@
       <x:c r="E8" s="16"/>
       <x:c r="F8" s="16"/>
       <x:c r="I8" s="22" t="str">
-        <x:v>nhánh validation rejected reset về upload, còn retry API backend được đánh dấu chưa nối UI</x:v>
+        <x:v>không có mặt, nhiều mặt hoặc detector lỗi đều quay lại chọn ảnh và không gọi API tạo sticker</x:v>
       </x:c>
       <x:c r="J8" s="22"/>
       <x:c r="K8" s="22"/>
@@ -1165,7 +1180,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="28" t="str">
-        <x:v>Happy path và nhánh rejected của CTA Thử Lại Ngay trong UI hiện tại.</x:v>
+        <x:v>đúng một mặt tiếp tục auth, job, polling và gallery</x:v>
       </x:c>
       <x:c r="B18" s="28"/>
       <x:c r="C18" s="28"/>
@@ -1173,7 +1188,7 @@
       <x:c r="E18" s="28"/>
       <x:c r="F18" s="28"/>
       <x:c r="I18" s="34" t="str">
-        <x:v>Happy path và nhánh rejected của CTA Thử Lại Ngay trong UI hiện tại.</x:v>
+        <x:v>User journey mới: ảnh chỉ đi tới xác thực và tạo job sau khi detector trả đúng một khuôn mặt.</x:v>
       </x:c>
       <x:c r="J18" s="34"/>
       <x:c r="K18" s="34"/>
@@ -1259,7 +1274,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="43" t="str">
-        <x:v>Luồng UI thực tế trên kien_v5, gồm auth, polling và rejected state
+        <x:v>Face preflight cục bộ đứng trước job và mọi image call trả phí
 Implemented  •  Inferred  •  Gap/Risk  •  Recommended</x:v>
       </x:c>
       <x:c r="B28" s="43"/>
@@ -1342,7 +1357,7 @@
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="A42" s="45" t="str">
-        <x:v>Hình GS-DOC-02 — User journey và nhánh phục hồi. Happy path và nhánh rejected của CTA Thử Lại Ngay trong UI hiện tại.</x:v>
+        <x:v>Hình GS-DOC-02 — User journey và nhánh phục hồi. User journey mới: ảnh chỉ đi tới xác thực và tạo job sau khi detector trả đúng một khuôn mặt.</x:v>
       </x:c>
       <x:c r="B42" s="45"/>
       <x:c r="C42" s="45"/>
@@ -1360,7 +1375,7 @@
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="49" t="str">
-        <x:v>Mô tả sơ đồ: Luồng từ chọn ảnh, xác thực, tạo job, polling đến gallery; nhánh validation rejected reset về upload, còn retry API backend được đánh dấu chưa nối UI.</x:v>
+        <x:v>Mô tả sơ đồ: Luồng chọn ảnh qua Web Worker MediaPipe; không có mặt, nhiều mặt hoặc detector lỗi đều quay lại chọn ảnh và không gọi API tạo sticker; đúng một mặt tiếp tục auth, job, polling và gallery.</x:v>
       </x:c>
       <x:c r="B44" s="49"/>
       <x:c r="C44" s="49"/>
@@ -1378,7 +1393,7 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="51" t="str">
-        <x:v>Nguồn: frontend/src/App.tsx; frontend/src/hooks/useStickerGenerator.ts; frontend/src/services/stickerService.ts  •  kien_v5 @ c09e26a  •  2026-08-09</x:v>
+        <x:v>Nguồn: frontend/src/components/upload/ImageUploader.tsx; frontend/src/hooks/useImageUpload.ts; frontend/src/services/faceDetectionService.ts  •  kien_v5 @ 4d23b9a  •  2026-08-10</x:v>
       </x:c>
       <x:c r="B46" s="51"/>
       <x:c r="C46" s="51"/>
@@ -1413,7 +1428,7 @@
   <x:printOptions horizontalCentered="1"/>
   <x:pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e06b7d628f64a7f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4db8f761ead047d3"/>
 </x:worksheet>
 </file>
 
@@ -1448,7 +1463,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -1597,7 +1612,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a92534101ce4b39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d06cfe21d514421"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1633,7 +1648,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -1760,7 +1775,204 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff18b8e3b1db4cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f7c6744fd1143c9"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="53" t="str">
+        <x:v>02  /  Product Requirements Document</x:v>
+      </x:c>
+      <x:c r="B1" s="53"/>
+      <x:c r="C1" s="53"/>
+      <x:c r="D1" s="53"/>
+      <x:c r="E1" s="53"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="56" t="str">
+        <x:v>Yêu cầu sản phẩm cho preflight đúng một khuôn mặt chạy cục bộ và không phát sinh chi phí</x:v>
+      </x:c>
+      <x:c r="B2" s="56"/>
+      <x:c r="C2" s="56"/>
+      <x:c r="D2" s="56"/>
+      <x:c r="E2" s="56"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="57" t="str">
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
+      </x:c>
+      <x:c r="B3" s="57"/>
+      <x:c r="C3" s="57"/>
+      <x:c r="D3" s="57"/>
+      <x:c r="E3" s="57"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="58" t="str">
+        <x:v>AS-BUILT • Nội dung viết từ source hiện tại; bộ mẫu chỉ cung cấp cấu trúc trình bày.</x:v>
+      </x:c>
+      <x:c r="B4" s="58"/>
+      <x:c r="C4" s="58"/>
+      <x:c r="D4" s="58"/>
+      <x:c r="E4" s="58"/>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="64" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B6" s="64" t="str">
+        <x:v>Requirement</x:v>
+      </x:c>
+      <x:c r="C6" s="64" t="str">
+        <x:v>Acceptance</x:v>
+      </x:c>
+      <x:c r="D6" s="64" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E6" s="64" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A7" s="69" t="str">
+        <x:v>FG-01</x:v>
+      </x:c>
+      <x:c r="B7" s="69" t="str">
+        <x:v>Chỉ accept detections.length = 1</x:v>
+      </x:c>
+      <x:c r="C7" s="69" t="str">
+        <x:v>0 reject; 1 verified; &gt;1 reject</x:v>
+      </x:c>
+      <x:c r="D7" s="69" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="E7" s="69" t="str">
+        <x:v>useImageUpload.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A8" s="70" t="str">
+        <x:v>FG-02</x:v>
+      </x:c>
+      <x:c r="B8" s="70" t="str">
+        <x:v>Không gửi ảnh ra ngoài trong preflight</x:v>
+      </x:c>
+      <x:c r="C8" s="70" t="str">
+        <x:v>Worker xử lý ImageBitmap local</x:v>
+      </x:c>
+      <x:c r="D8" s="70" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="E8" s="70" t="str">
+        <x:v>faceDetector.worker.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A9" s="69" t="str">
+        <x:v>FG-03</x:v>
+      </x:c>
+      <x:c r="B9" s="69" t="str">
+        <x:v>Không GPU/paid vision API</x:v>
+      </x:c>
+      <x:c r="C9" s="69" t="str">
+        <x:v>CPU/WASM; không API key</x:v>
+      </x:c>
+      <x:c r="D9" s="69" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="E9" s="69" t="str">
+        <x:v>public/models/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" hidden="0" customHeight="1">
+      <x:c r="A10" s="70" t="str">
+        <x:v>FG-04</x:v>
+      </x:c>
+      <x:c r="B10" s="70" t="str">
+        <x:v>Fail closed khi unsupported/timeout</x:v>
+      </x:c>
+      <x:c r="C10" s="70" t="str">
+        <x:v>Không có preview/file hợp lệ và không Generate</x:v>
+      </x:c>
+      <x:c r="D10" s="70" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="E10" s="70" t="str">
+        <x:v>faceDetectionService.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A11" s="69" t="str">
+        <x:v>FG-05</x:v>
+      </x:c>
+      <x:c r="B11" s="69" t="str">
+        <x:v>Không đổi generation contract</x:v>
+      </x:c>
+      <x:c r="C11" s="69" t="str">
+        <x:v>onStartGeneration chỉ chạy sau verified</x:v>
+      </x:c>
+      <x:c r="D11" s="69" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="E11" s="69" t="str">
+        <x:v>ImageUploader.tsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A12" s="70" t="str">
+        <x:v>FG-06</x:v>
+      </x:c>
+      <x:c r="B12" s="70" t="str">
+        <x:v>Authoritative backend check</x:v>
+      </x:c>
+      <x:c r="C12" s="70" t="str">
+        <x:v>Direct API cũng bị semantic gate</x:v>
+      </x:c>
+      <x:c r="D12" s="70" t="str">
+        <x:v>Gap</x:v>
+      </x:c>
+      <x:c r="E12" s="70" t="str">
+        <x:v>Chưa có server detector</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A13" s="69" t="str">
+        <x:v>FG-07</x:v>
+      </x:c>
+      <x:c r="B13" s="69" t="str">
+        <x:v>Metrics</x:v>
+      </x:c>
+      <x:c r="C13" s="69" t="str">
+        <x:v>Latency/accept/reject/error rate</x:v>
+      </x:c>
+      <x:c r="D13" s="69" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E13" s="69" t="str">
+        <x:v>Chưa có telemetry</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+    <x:mergeCell ref="A4:E4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bf00ba1224c4216"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1790,7 +2002,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -1887,7 +2099,7 @@
         <x:v>75 backend tests; frontend lint/build đạt</x:v>
       </x:c>
       <x:c r="C13" s="69" t="str">
-        <x:v>Kiểm tra cục bộ 2026-08-09</x:v>
+        <x:v>Kiểm tra cục bộ 2026-08-10</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1899,7 +2111,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7553add357084724"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R838552e41c7a4aa0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1910,11 +2122,11 @@
   <x:cols>
     <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="33" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="39" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1944,7 +2156,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -2356,6 +2568,32 @@
         <x:v>Gap</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A21" s="69" t="str">
+        <x:v>PRD-015</x:v>
+      </x:c>
+      <x:c r="B21" s="69" t="str">
+        <x:v>Input gate</x:v>
+      </x:c>
+      <x:c r="C21" s="69" t="str">
+        <x:v>Kiểm tra đúng một khuôn mặt trong browser trước generation</x:v>
+      </x:c>
+      <x:c r="D21" s="69" t="str">
+        <x:v>0 mặt reject; 1 mặt verified; &gt;1 mặt reject; failure fail closed</x:v>
+      </x:c>
+      <x:c r="E21" s="69" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F21" s="72" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="G21" s="69" t="str">
+        <x:v>frontend/src/hooks/useImageUpload.ts; frontend/src/workers/faceDetector.worker.ts</x:v>
+      </x:c>
+      <x:c r="H21" s="69" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -2363,14 +2601,14 @@
     <x:mergeCell ref="A3:H3"/>
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E7:E20">
+  <x:conditionalFormatting sqref="E7:E21">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="P1"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="P2"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12be1c54ad044753"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bc5da8a95d344d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2406,7 +2644,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -2550,7 +2788,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9974bd964eef4c29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R869d6b9cf2e24461"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2583,7 +2821,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -2746,7 +2984,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R513700e29286483a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42655b2a44a4166"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2782,7 +3020,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -2926,7 +3164,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ee26fe6eb854254"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b7025f8066b4c6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2951,7 +3189,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="56" t="str">
-        <x:v>Phân bố 14 yêu cầu theo mức triển khai từ source audit</x:v>
+        <x:v>Phân bố 15 yêu cầu theo mức triển khai từ source audit</x:v>
       </x:c>
       <x:c r="B2" s="56"/>
       <x:c r="C2" s="56"/>
@@ -2960,7 +3198,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -2992,8 +3230,8 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B7" s="69" t="n">
-        <x:f>COUNTIF(Requirements!$H$7:$H$20,A7)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIF(Requirements!$H$7:$H$21,A7)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="69" t="str">
         <x:v>Có code path và không ghi nhận gap trực tiếp</x:v>
@@ -3004,7 +3242,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B8" s="70" t="n">
-        <x:f>COUNTIF(Requirements!$H$7:$H$20,A8)</x:f>
+        <x:f>COUNTIF(Requirements!$H$7:$H$21,A8)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C8" s="70" t="str">
@@ -3016,7 +3254,7 @@
         <x:v>Gap</x:v>
       </x:c>
       <x:c r="B9" s="69" t="n">
-        <x:f>COUNTIF(Requirements!$H$7:$H$20,A9)</x:f>
+        <x:f>COUNTIF(Requirements!$H$7:$H$21,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="69" t="str">
@@ -3031,9 +3269,9 @@
     <x:mergeCell ref="A4:E4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffe7494fdae04e07"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2a42469c1524829"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe40014051c342bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc748aff7693048c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3066,7 +3304,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -3159,7 +3397,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720683b431dc4bee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raacb9a5cf4414de1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3195,7 +3433,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="57" t="str">
-        <x:v>GS-DOC-02  •  kien_v5 @ c09e26a  •  2026-08-09  •  Current + gaps</x:v>
+        <x:v>GS-DOC-02  •  kien_v5 @ 4d23b9a  •  2026-08-10  •  Current + gaps</x:v>
       </x:c>
       <x:c r="B3" s="57"/>
       <x:c r="C3" s="57"/>
@@ -3322,7 +3560,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32816da4361f49f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18206161b496485d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>